<commit_message>
added seminar speakers info
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29912"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29917"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="362" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C389BF6-7B71-4379-89DC-61D8349F7487}"/>
+  <xr:revisionPtr revIDLastSave="379" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46B3E0D4-3D9E-48F0-9E3C-83567FBEBCA1}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="427">
   <si>
     <t>Fill in as much of the green boxes as possible. Ideally, this would be before you have finished your visitors travel dates (just to avoid double booking).</t>
   </si>
@@ -1219,6 +1219,13 @@
     <t>Carl Scarrott</t>
   </si>
   <si>
+    <t>Bayes-ically Fair:  Bayesian Ranking of Olympic Medal Performances</t>
+  </si>
+  <si>
+    <t>Evaluating a country's sporting success can provide insight into its decision-making and the infrastructure used to develop athletic talent. The Olympic Games serve as a global benchmark, yet conventional medal tables can be overly influenced by population size or highly variable, particularly for smaller nations where outcomes are more affected by stochastic fluctuations.
+We propose a Bayesian ranking scheme to rank the performance of National Olympic Committees by inferring an underlying `long-run' medals-to-population rate. The approach applies shrinkage to stabilise estimates for small-population countries while leaving large-population countries comparatively unchanged. The Bayesian framework yields posterior distributions over both the inferred medals-per-capita performance and the induced ranks, providing a principled measure of uncertainty in each country's ranking position.</t>
+  </si>
+  <si>
     <t>https://scholar.google.com/citations?user=kRgtZZcAAAAJ&amp;hl=en</t>
   </si>
   <si>
@@ -1228,10 +1235,16 @@
     <t>Andrew Keane</t>
   </si>
   <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Alan Demlow</t>
+  </si>
+  <si>
+    <t>Texas A&amp;M</t>
+  </si>
+  <si>
     <t>Open</t>
-  </si>
-  <si>
-    <t>May</t>
   </si>
   <si>
     <t>This is a just a place for those who are interested but that dont have a specific date in mind. (Ideally, a couple of these are people that we could invite with relatively short notice to fill missing slots.)</t>
@@ -6958,7 +6971,7 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1">
       <c r="A12" s="75">
         <v>46128</v>
       </c>
@@ -6986,17 +6999,17 @@
         <v>78</v>
       </c>
       <c r="I12" s="98" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="J12" s="98" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="K12" s="102" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="L12" s="5"/>
       <c r="M12" s="24" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="N12" s="16"/>
       <c r="O12" s="35"/>
@@ -7028,7 +7041,7 @@
         <v>13</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>73</v>
@@ -7059,9 +7072,36 @@
       <c r="Y13" s="13"/>
     </row>
     <row r="14" spans="1:25">
-      <c r="A14" s="26"/>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
+      <c r="A14" s="26">
+        <v>46156</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>190</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>375</v>
+      </c>
+      <c r="D14" t="s">
+        <v>278</v>
+      </c>
+      <c r="E14">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>376</v>
+      </c>
+      <c r="G14" t="s">
+        <v>377</v>
+      </c>
+      <c r="H14" t="s">
+        <v>40</v>
+      </c>
+      <c r="I14" t="s">
+        <v>363</v>
+      </c>
+      <c r="J14" t="s">
+        <v>363</v>
+      </c>
       <c r="X14" s="20"/>
       <c r="Y14" s="18"/>
     </row>
@@ -7244,7 +7284,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="G3" s="14" t="s">
         <v>363</v>
@@ -7295,7 +7335,7 @@
         <v>3</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>363</v>
@@ -7346,7 +7386,7 @@
         <v>5</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>363</v>
@@ -7401,7 +7441,7 @@
         <v>7</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>363</v>
@@ -7452,7 +7492,7 @@
         <v>9</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="G7" s="14" t="s">
         <v>363</v>
@@ -7501,7 +7541,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="G8" s="14" t="s">
         <v>363</v>
@@ -7539,7 +7579,7 @@
         <v>190</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D9" s="27" t="s">
         <v>278</v>
@@ -7548,7 +7588,7 @@
         <v>13</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>363</v>
@@ -7626,23 +7666,23 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="55" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B2" s="54" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="136" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="B3" s="137"/>
       <c r="C3" s="138" t="s">
@@ -7651,7 +7691,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="B4" s="52"/>
       <c r="C4" s="50" t="s">
@@ -7660,19 +7700,19 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="52" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="B5" s="52"/>
       <c r="C5" s="50" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="52" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="B6" s="52" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="C6" s="50" t="s">
         <v>87</v>
@@ -7680,10 +7720,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="52" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="B7" s="52" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="C7" s="50" t="s">
         <v>87</v>
@@ -7691,10 +7731,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="52" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="C8" s="50" t="s">
         <v>101</v>
@@ -7702,75 +7742,75 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="52" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="B9" s="52"/>
       <c r="C9" s="50"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="52" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="52" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B11" s="52" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="52" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="B12" s="52" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="52" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="B13" s="52" t="s">
+        <v>403</v>
+      </c>
+      <c r="C13" s="50" t="s">
         <v>399</v>
-      </c>
-      <c r="C13" s="50" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="52" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="52" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -7778,10 +7818,10 @@
         <v>321</v>
       </c>
       <c r="B16" s="137" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="C16" s="139" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7789,18 +7829,18 @@
         <v>346</v>
       </c>
       <c r="B17" s="137" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="C17" s="139" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="52" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="C18" s="50" t="s">
         <v>87</v>
@@ -7808,21 +7848,21 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="53" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="B19" s="53" t="s">
         <v>230</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B20" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>
@@ -7849,10 +7889,10 @@
         <v>3</v>
       </c>
       <c r="B1" s="131" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C1" s="130" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -7863,7 +7903,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="170" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="F2" s="75"/>
       <c r="G2" s="77"/>
@@ -7880,7 +7920,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="170" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="F3" s="75"/>
       <c r="G3" s="2"/>
@@ -7897,7 +7937,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="170" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="F4" s="75"/>
       <c r="G4" s="2"/>
@@ -7914,7 +7954,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="170" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="F5" s="75"/>
       <c r="G5" s="2"/>
@@ -7931,7 +7971,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="134" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="F6" s="75"/>
       <c r="G6" s="2"/>
@@ -7948,7 +7988,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="134" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="F7" s="75"/>
       <c r="G7" s="2"/>
@@ -7965,7 +8005,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="134" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="F8" s="75"/>
       <c r="G8" s="2"/>
@@ -7982,7 +8022,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="134" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="F9" s="75"/>
       <c r="G9" s="2"/>
@@ -7999,7 +8039,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="134" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="F10" s="75"/>
       <c r="G10" s="2"/>
@@ -8016,7 +8056,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="134" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -8029,7 +8069,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="134" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -8042,7 +8082,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="134" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -8055,7 +8095,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="134" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -8104,12 +8144,12 @@
   <sheetData>
     <row r="2" spans="1:9" ht="23.25">
       <c r="A2" s="91" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="18.75">
       <c r="A3" s="79" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="35.25">
@@ -8135,7 +8175,7 @@
         <v>9</v>
       </c>
       <c r="H5" s="82" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="I5" s="81" t="s">
         <v>11</v>
@@ -8235,7 +8275,7 @@
         <v>198</v>
       </c>
       <c r="D9" s="94" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="E9" s="94">
         <v>8</v>
@@ -8297,7 +8337,7 @@
         <v>10</v>
       </c>
       <c r="F11" s="87" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="G11" s="87" t="s">
         <v>68</v>
@@ -8353,7 +8393,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="87" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="G13" s="87"/>
       <c r="H13" s="87"/>
@@ -8376,7 +8416,7 @@
         <v>13</v>
       </c>
       <c r="F14" s="90" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="G14" s="90" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
added seminar title and abs
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="379" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46B3E0D4-3D9E-48F0-9E3C-83567FBEBCA1}"/>
+  <xr:revisionPtr revIDLastSave="384" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCC967C4-95DF-48D7-8A3B-9B5914B78022}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="429">
   <si>
     <t>Fill in as much of the green boxes as possible. Ideally, this would be before you have finished your visitors travel dates (just to avoid double booking).</t>
   </si>
@@ -1198,7 +1198,10 @@
     <t xml:space="preserve">Chris Howland </t>
   </si>
   <si>
-    <t>TBC</t>
+    <t>Convection and phase changes in environmental flows</t>
+  </si>
+  <si>
+    <t>Many processes in the climate system can be related to the coupling of fluid convection and thermodynamic phase changes, from ice-ocean interactions in polar regions to the formation and evolution of clouds in the atmosphere. In this talk, I will discuss some recent work aimed at understanding the fundamental interactions between convection and phase changes in simple systems, with a focus on the effects of turbulence on ice melting. Firstly, motivated by the flows beside marine-terminating glaciers, I will describe work focused on understanding boundary layers in turbulent convection at vertical walls. I focus on the complexities introduced by a high Prandtl number (relevant to seawater) and the effect of an ambient flow, where a transition between buoyancy-driven and shear-driven boundary layers occurs. Secondly, I will outline a newly-developed immersed boundary technique for simulating melting objects in turbulent flows, which reveals the subtle effects that the free motion of melting ice objects can introduce.</t>
   </si>
   <si>
     <t>Michel Destrade</t>
@@ -1233,6 +1236,9 @@
   </si>
   <si>
     <t>Andrew Keane</t>
+  </si>
+  <si>
+    <t>TBC</t>
   </si>
   <si>
     <t>May</t>
@@ -6871,7 +6877,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:25" ht="15" customHeight="1">
       <c r="A10" s="75">
         <v>46120</v>
       </c>
@@ -6902,7 +6908,7 @@
         <v>363</v>
       </c>
       <c r="J10" s="98" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K10" s="102"/>
       <c r="L10" s="5"/>
@@ -6937,7 +6943,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>195</v>
@@ -6946,17 +6952,17 @@
         <v>87</v>
       </c>
       <c r="I11" s="98" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="J11" s="98" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K11" s="102" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="24" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="N11" s="16"/>
       <c r="O11" s="35"/>
@@ -6990,7 +6996,7 @@
         <v>12</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>195</v>
@@ -6999,17 +7005,17 @@
         <v>78</v>
       </c>
       <c r="I12" s="98" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J12" s="98" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K12" s="102" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="L12" s="5"/>
       <c r="M12" s="24" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="N12" s="16"/>
       <c r="O12" s="35"/>
@@ -7041,7 +7047,7 @@
         <v>13</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>73</v>
@@ -7050,10 +7056,10 @@
         <v>95</v>
       </c>
       <c r="I13" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="J13" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="K13" s="102"/>
       <c r="L13" s="5"/>
@@ -7079,7 +7085,7 @@
         <v>190</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D14" t="s">
         <v>278</v>
@@ -7088,19 +7094,19 @@
         <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="G14" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H14" t="s">
         <v>40</v>
       </c>
       <c r="I14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="J14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="X14" s="20"/>
       <c r="Y14" s="18"/>
@@ -7284,19 +7290,19 @@
         <v>1</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="H3" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="I3" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="J3" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="K3" s="73"/>
       <c r="L3" s="40"/>
@@ -7335,19 +7341,19 @@
         <v>3</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="I4" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="J4" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="K4" s="102"/>
       <c r="L4" s="5"/>
@@ -7386,19 +7392,19 @@
         <v>5</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="I5" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="J5" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="K5" s="102"/>
       <c r="L5" s="5"/>
@@ -7441,19 +7447,19 @@
         <v>7</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="H6" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="I6" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="J6" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="K6" s="102"/>
       <c r="L6" s="5"/>
@@ -7492,19 +7498,19 @@
         <v>9</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="I7" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="J7" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="K7" s="102"/>
       <c r="L7" s="5"/>
@@ -7541,19 +7547,19 @@
         <v>11</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="I8" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="J8" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="K8" s="102"/>
       <c r="L8" s="5"/>
@@ -7579,7 +7585,7 @@
         <v>190</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D9" s="27" t="s">
         <v>278</v>
@@ -7588,19 +7594,19 @@
         <v>13</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="I9" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="J9" s="98" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
       <c r="K9" s="102"/>
       <c r="L9" s="5"/>
@@ -7666,23 +7672,23 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="55" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B2" s="54" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="136" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B3" s="137"/>
       <c r="C3" s="138" t="s">
@@ -7691,7 +7697,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B4" s="52"/>
       <c r="C4" s="50" t="s">
@@ -7700,19 +7706,19 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="52" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B5" s="52"/>
       <c r="C5" s="50" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="52" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B6" s="52" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C6" s="50" t="s">
         <v>87</v>
@@ -7720,10 +7726,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="52" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B7" s="52" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C7" s="50" t="s">
         <v>87</v>
@@ -7731,10 +7737,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="52" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="C8" s="50" t="s">
         <v>101</v>
@@ -7742,75 +7748,75 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="52" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B9" s="52"/>
       <c r="C9" s="50"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="52" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="52" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B11" s="52" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="52" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B12" s="52" t="s">
+        <v>403</v>
+      </c>
+      <c r="C12" s="50" t="s">
         <v>401</v>
-      </c>
-      <c r="C12" s="50" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="52" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B13" s="52" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="52" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="52" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -7818,10 +7824,10 @@
         <v>321</v>
       </c>
       <c r="B16" s="137" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="C16" s="139" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7829,18 +7835,18 @@
         <v>346</v>
       </c>
       <c r="B17" s="137" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="C17" s="139" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="52" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C18" s="50" t="s">
         <v>87</v>
@@ -7848,21 +7854,21 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="53" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B19" s="53" t="s">
         <v>230</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B20" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -7889,10 +7895,10 @@
         <v>3</v>
       </c>
       <c r="B1" s="131" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C1" s="130" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -7903,7 +7909,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="170" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="F2" s="75"/>
       <c r="G2" s="77"/>
@@ -7920,7 +7926,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="170" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F3" s="75"/>
       <c r="G3" s="2"/>
@@ -7937,7 +7943,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="170" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="F4" s="75"/>
       <c r="G4" s="2"/>
@@ -7954,7 +7960,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="170" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F5" s="75"/>
       <c r="G5" s="2"/>
@@ -7971,7 +7977,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="134" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="F6" s="75"/>
       <c r="G6" s="2"/>
@@ -7988,7 +7994,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="134" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="F7" s="75"/>
       <c r="G7" s="2"/>
@@ -8005,7 +8011,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="134" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="F8" s="75"/>
       <c r="G8" s="2"/>
@@ -8022,7 +8028,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="134" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="F9" s="75"/>
       <c r="G9" s="2"/>
@@ -8039,7 +8045,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="134" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="F10" s="75"/>
       <c r="G10" s="2"/>
@@ -8056,7 +8062,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="134" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -8069,7 +8075,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="134" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -8082,7 +8088,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="134" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -8095,7 +8101,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="134" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -8144,12 +8150,12 @@
   <sheetData>
     <row r="2" spans="1:9" ht="23.25">
       <c r="A2" s="91" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="18.75">
       <c r="A3" s="79" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="35.25">
@@ -8175,7 +8181,7 @@
         <v>9</v>
       </c>
       <c r="H5" s="82" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="I5" s="81" t="s">
         <v>11</v>
@@ -8205,7 +8211,7 @@
       </c>
       <c r="H6" s="85"/>
       <c r="I6" s="84" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="18.75">
@@ -8275,7 +8281,7 @@
         <v>198</v>
       </c>
       <c r="D9" s="94" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E9" s="94">
         <v>8</v>
@@ -8290,7 +8296,7 @@
         <v>206</v>
       </c>
       <c r="I9" s="86" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="18.75">
@@ -8337,14 +8343,14 @@
         <v>10</v>
       </c>
       <c r="F11" s="87" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="G11" s="87" t="s">
         <v>68</v>
       </c>
       <c r="H11" s="87"/>
       <c r="I11" s="86" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="18.75">
@@ -8373,7 +8379,7 @@
         <v>31</v>
       </c>
       <c r="I12" s="86" t="s">
-        <v>363</v>
+        <v>376</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="18.75">
@@ -8393,7 +8399,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="87" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="G13" s="87"/>
       <c r="H13" s="87"/>
@@ -8416,7 +8422,7 @@
         <v>13</v>
       </c>
       <c r="F14" s="90" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="G14" s="90" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
added speaker for JG
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30015"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="414" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A2A1BF9-C7FF-45AC-8963-FB752E233DAB}"/>
+  <xr:revisionPtr revIDLastSave="416" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8ABB13C-981A-4743-ABF0-CA69466D205E}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1039" uniqueCount="438">
   <si>
     <t>Fill in as much of the green boxes as possible. Ideally, this would be before you have finished your visitors travel dates (just to avoid double booking).</t>
   </si>
@@ -1238,24 +1238,45 @@
     <t>Andrew Keane</t>
   </si>
   <si>
+    <t>Fragmented tipping of the Atlantic Meridional Ocean Circulation</t>
+  </si>
+  <si>
+    <t>The tipping of the Atlantic Meridional Overturning Circulation (AMOC) to a ‘shutdown’ state due to changes in the freshwater forcing of the ocean is of particular interest and concern due to its widespread ramifications, including a dramatic climatic shift for much of Europe. A clear understanding of how such a shutdown would unfold requires analyses of models from across the complexity spectrum. For example, detailed simulations of sophisticated Earth System Models have identified scenarios of ‘fragmented’ tipping towards a complete shutdown of AMOC, in which deep-water formation first ceases in the Labrador Sea before ceasing in the Nordic Seas. Here, we study a simple ocean box model with two polar boxes designed to represent deep-water formation at these two distinct sites. A bifurcation analysis reveals how, depending on the differences of freshwater and thermal forcing between the two polar boxes, transitions to ‘partial shutdown’ states are possible. Our results shed light on the nature of the tipping of AMOC and clarify dynamical features observed in more sophisticated models.</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Florian Faucher</t>
+  </si>
+  <si>
+    <t>University of Pau and Pays de l’Adour</t>
+  </si>
+  <si>
+    <t>Romina Gaburro</t>
+  </si>
+  <si>
+    <t>Quantitative inverse wave problem for passive imaging using cross-correlation data.</t>
+  </si>
+  <si>
+    <t>We investigate the quantitative reconstruction of physical properties in the context of passive imaging, where ambient wavefields are used to probe a medium. These ambient signals correspond to oscillations of the system generated by stochastic events. We discuss in particular  helioseismology, where satellites observe solar oscillations that are driven by turbulent convective motion. Considering the data as a superposition of waves generated by stochastic sources, the expected value of the cross-correlation between signals is related to the deterministic Green's function. The inverse wave problem is then formulated through an iterative minimization procedure, in which the gradient of the misfit functional is computed via the adjoint-state method. We focus on time-harmonic acoustic wave propagation and carry out synthetic experiments, comparing inversions based on cross-correlation data with those using direct wavefield measurements in the configuration of active-source acquisitions.</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/citations?user=KKQ8FvkAAAAJ&amp;hl=en</t>
+  </si>
+  <si>
+    <t>https://ffaucher.gitlab.io/cv/</t>
+  </si>
+  <si>
+    <t>Alan Demlow</t>
+  </si>
+  <si>
+    <t>Texas A&amp;M</t>
+  </si>
+  <si>
     <t>TBC</t>
   </si>
   <si>
-    <t>May</t>
-  </si>
-  <si>
-    <t>Florian Faucher</t>
-  </si>
-  <si>
-    <t>University of Pau and Pays de l’Adour</t>
-  </si>
-  <si>
-    <t>Alan Demlow</t>
-  </si>
-  <si>
-    <t>Texas A&amp;M</t>
-  </si>
-  <si>
     <t>Open</t>
   </si>
   <si>
@@ -1401,21 +1422,6 @@
   </si>
   <si>
     <t>Leornard Henckel</t>
-  </si>
-  <si>
-    <t>Romina Gaburro</t>
-  </si>
-  <si>
-    <t>Quantitative inverse wave problem for passive imaging using cross-correlation data.</t>
-  </si>
-  <si>
-    <t>We investigate the quantitative reconstruction of physical properties in the context of passive imaging, where ambient wavefields are used to probe a medium. These ambient signals correspond to oscillations of the system generated by stochastic events. We discuss in particular  helioseismology, where satellites observe solar oscillations that are driven by turbulent convective motion. Considering the data as a superposition of waves generated by stochastic sources, the expected value of the cross-correlation between signals is related to the deterministic Green's function. The inverse wave problem is then formulated through an iterative minimization procedure, in which the gradient of the misfit functional is computed via the adjoint-state method. We focus on time-harmonic acoustic wave propagation and carry out synthetic experiments, comparing inversions based on cross-correlation data with those using direct wavefield measurements in the configuration of active-source acquisitions.</t>
-  </si>
-  <si>
-    <t>https://ffaucher.gitlab.io/cv/</t>
-  </si>
-  <si>
-    <t>https://scholar.google.com/citations?user=KKQ8FvkAAAAJ&amp;hl=en</t>
   </si>
 </sst>
 </file>
@@ -1425,7 +1431,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2283,9 +2289,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2323,7 +2329,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2429,7 +2435,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2571,7 +2577,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2580,7 +2586,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7958562-D4BB-4776-9668-682A6F2E2AD0}">
   <dimension ref="A1:Y20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="11.140625" customWidth="1"/>
@@ -2605,7 +2611,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2616,7 +2622,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="30">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2693,7 +2699,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="13.5" customHeight="1">
       <c r="A3" s="2">
         <v>45317</v>
       </c>
@@ -2760,7 +2766,7 @@
       <c r="X3" s="13"/>
       <c r="Y3" s="13"/>
     </row>
-    <row r="4" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="13.5" customHeight="1">
       <c r="A4" s="2">
         <v>45323</v>
       </c>
@@ -2823,7 +2829,7 @@
       <c r="X4" s="13"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25">
       <c r="A5" s="2">
         <v>45324</v>
       </c>
@@ -2884,7 +2890,7 @@
       <c r="X5" s="13"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="12.75" customHeight="1">
       <c r="A6" s="2">
         <v>45331</v>
       </c>
@@ -2951,7 +2957,7 @@
       <c r="X6" s="13"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25">
       <c r="A7" s="2">
         <v>45338</v>
       </c>
@@ -3020,7 +3026,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="15" customHeight="1">
       <c r="A8" s="2">
         <v>45345</v>
       </c>
@@ -3087,7 +3093,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="16.5" customHeight="1">
       <c r="A9" s="2">
         <v>45359</v>
       </c>
@@ -3140,7 +3146,7 @@
       <c r="X9" s="13"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25">
       <c r="A10" s="2">
         <v>45366</v>
       </c>
@@ -3209,7 +3215,7 @@
       <c r="X10" s="13"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15" customHeight="1">
       <c r="A11" s="2">
         <v>45379</v>
       </c>
@@ -3270,7 +3276,7 @@
       <c r="X11" s="13"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="13.5" customHeight="1">
       <c r="A12" s="2">
         <v>45386</v>
       </c>
@@ -3333,7 +3339,7 @@
       <c r="X12" s="13"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="16.5" customHeight="1">
       <c r="A13" s="2">
         <v>45387</v>
       </c>
@@ -3402,7 +3408,7 @@
       <c r="X13" s="13"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1">
       <c r="A14" s="2">
         <v>45394</v>
       </c>
@@ -3463,7 +3469,7 @@
       <c r="X14" s="13"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="17.25" customHeight="1">
       <c r="A15" s="2">
         <v>45398</v>
       </c>
@@ -3532,7 +3538,7 @@
       <c r="X15" s="13"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25">
       <c r="A16" s="2">
         <v>45401</v>
       </c>
@@ -3595,7 +3601,7 @@
       <c r="X16" s="18"/>
       <c r="Y16" s="18"/>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25">
       <c r="A17" s="4">
         <v>45421</v>
       </c>
@@ -3666,7 +3672,7 @@
       <c r="X17" s="18"/>
       <c r="Y17" s="18"/>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25">
       <c r="A18" s="26">
         <v>45474</v>
       </c>
@@ -3717,7 +3723,7 @@
       <c r="X18" s="18"/>
       <c r="Y18" s="18"/>
     </row>
-    <row r="19" spans="1:25" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:25" ht="17.25" customHeight="1" thickBot="1">
       <c r="A19" s="26">
         <v>45505</v>
       </c>
@@ -3768,7 +3774,7 @@
       <c r="X19" s="18"/>
       <c r="Y19" s="18"/>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25">
       <c r="A20" s="26"/>
       <c r="B20" s="26"/>
       <c r="C20" s="26"/>
@@ -3810,7 +3816,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="11.140625" customWidth="1"/>
@@ -3835,7 +3841,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3846,7 +3852,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" ht="30.75" thickBot="1">
       <c r="A2" s="145" t="s">
         <v>3</v>
       </c>
@@ -3923,7 +3929,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15" customHeight="1">
       <c r="A3" s="2">
         <v>45548</v>
       </c>
@@ -3988,7 +3994,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15" customHeight="1">
       <c r="A4" s="2">
         <v>45555</v>
       </c>
@@ -4037,7 +4043,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="15" customHeight="1">
       <c r="A5" s="2">
         <v>45562</v>
       </c>
@@ -4086,7 +4092,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15" customHeight="1">
       <c r="A6" s="2">
         <v>45576</v>
       </c>
@@ -4135,7 +4141,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="15" customHeight="1">
       <c r="A7" s="2">
         <v>45583</v>
       </c>
@@ -4184,7 +4190,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="15" customHeight="1">
       <c r="A8" s="2">
         <v>45596</v>
       </c>
@@ -4233,7 +4239,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="15" customHeight="1">
       <c r="A9" s="2">
         <v>45604</v>
       </c>
@@ -4282,7 +4288,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15" customHeight="1">
       <c r="A10" s="2">
         <v>45611</v>
       </c>
@@ -4331,7 +4337,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15" customHeight="1">
       <c r="A11" s="2">
         <v>45625</v>
       </c>
@@ -4380,7 +4386,7 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25" ht="15" customHeight="1" thickBot="1">
       <c r="A12" s="4">
         <v>45632</v>
       </c>
@@ -4437,20 +4443,20 @@
       <c r="X12" s="20"/>
       <c r="Y12" s="18"/>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25">
       <c r="A13" s="26"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
       <c r="D13" s="26"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25">
       <c r="A14" s="26"/>
       <c r="B14" s="26"/>
       <c r="C14" s="26"/>
       <c r="D14" s="26"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -4462,59 +4468,59 @@
       <c r="I29" s="61"/>
       <c r="J29" s="61"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10">
       <c r="A31" s="60"/>
       <c r="B31" s="60"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10">
       <c r="A32" s="60"/>
       <c r="B32" s="60"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2">
       <c r="A33" s="60"/>
       <c r="B33" s="60"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2">
       <c r="A34" s="60"/>
       <c r="B34" s="60"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2">
       <c r="A35" s="60"/>
       <c r="B35" s="60"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2">
       <c r="A36" s="60"/>
       <c r="B36" s="60"/>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2">
       <c r="A37" s="60"/>
       <c r="B37" s="60"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2">
       <c r="A38" s="60"/>
       <c r="B38" s="60"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2">
       <c r="A39" s="60"/>
       <c r="B39" s="60"/>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2">
       <c r="A40" s="60"/>
       <c r="B40" s="60"/>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2">
       <c r="A41" s="60"/>
       <c r="B41" s="60"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2">
       <c r="A42" s="60"/>
       <c r="B42" s="60"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2">
       <c r="A43" s="60"/>
       <c r="B43" s="60"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2">
       <c r="A44" s="60"/>
       <c r="B44" s="60"/>
     </row>
@@ -4543,7 +4549,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12299A9A-6C0C-4F92-957E-FBFCB6211744}">
   <dimension ref="A1:Y45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="5.85546875" bestFit="1" customWidth="1"/>
@@ -4571,7 +4577,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4582,7 +4588,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" ht="27.75" customHeight="1" thickBot="1">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -4659,7 +4665,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15" customHeight="1">
       <c r="A3" s="2">
         <v>45694</v>
       </c>
@@ -4711,7 +4717,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="14.25" customHeight="1">
       <c r="A4" s="2">
         <v>45708</v>
       </c>
@@ -4769,7 +4775,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="14.25" customHeight="1">
       <c r="A5" s="2">
         <v>45722</v>
       </c>
@@ -4825,7 +4831,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="16.5" customHeight="1">
       <c r="A6" s="2">
         <v>45735</v>
       </c>
@@ -4881,7 +4887,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="18" customHeight="1">
       <c r="A7" s="2">
         <v>45750</v>
       </c>
@@ -4935,7 +4941,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="16.5" customHeight="1">
       <c r="A8" s="2">
         <v>45751</v>
       </c>
@@ -4994,7 +5000,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1">
       <c r="A9" s="2">
         <v>45757</v>
       </c>
@@ -5056,7 +5062,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1">
       <c r="A10" s="2">
         <v>45758</v>
       </c>
@@ -5110,7 +5116,7 @@
       <c r="X10" s="20"/>
       <c r="Y10" s="18"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1">
       <c r="A11" s="4">
         <v>45764</v>
       </c>
@@ -5170,7 +5176,7 @@
       <c r="X11" s="35"/>
       <c r="Y11" s="35"/>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1">
       <c r="A12" s="4">
         <v>45771</v>
       </c>
@@ -5231,7 +5237,7 @@
       <c r="X12" s="35"/>
       <c r="Y12" s="35"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1">
       <c r="A13" s="2">
         <v>45785</v>
       </c>
@@ -5284,7 +5290,7 @@
       <c r="X13" s="35"/>
       <c r="Y13" s="35"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1">
       <c r="A14" s="4">
         <v>45799</v>
       </c>
@@ -5330,7 +5336,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1">
       <c r="A15" s="4">
         <v>45805</v>
       </c>
@@ -5364,101 +5370,101 @@
         <v>250</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1">
       <c r="A16" s="75"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2">
       <c r="A17" s="26"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2">
       <c r="A18" s="26"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2">
       <c r="A19" s="26"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2">
       <c r="A20" s="75"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2">
       <c r="A21" s="26"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2">
       <c r="A22" s="75"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2">
       <c r="A23" s="26"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2">
       <c r="A24" s="26"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2">
       <c r="A25" s="26"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2">
       <c r="A26" s="26"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2">
       <c r="A27" s="26"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2">
       <c r="A28" s="26"/>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2">
       <c r="B31" s="60"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2">
       <c r="A32" s="60"/>
       <c r="B32" s="60"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2">
       <c r="A33" s="60"/>
       <c r="B33" s="60"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2">
       <c r="A34" s="60"/>
       <c r="B34" s="60"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2">
       <c r="A35" s="60"/>
       <c r="B35" s="60"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2">
       <c r="A36" s="60"/>
       <c r="B36" s="60"/>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2">
       <c r="A37" s="60"/>
       <c r="B37" s="60"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2">
       <c r="A38" s="60"/>
       <c r="B38" s="60"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2">
       <c r="A39" s="60"/>
       <c r="B39" s="60"/>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2">
       <c r="A40" s="60"/>
       <c r="B40" s="60"/>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2">
       <c r="A41" s="60"/>
       <c r="B41" s="60"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2">
       <c r="A42" s="60"/>
       <c r="B42" s="60"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2">
       <c r="A43" s="60"/>
       <c r="B43" s="60"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2">
       <c r="A44" s="60"/>
       <c r="B44" s="60"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2">
       <c r="A45" s="60"/>
     </row>
   </sheetData>
@@ -5483,7 +5489,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{243C2AD8-98F5-4435-96A3-1C2CAB922825}">
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
@@ -5510,7 +5516,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5521,7 +5527,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="30">
       <c r="A2" s="78" t="s">
         <v>3</v>
       </c>
@@ -5598,7 +5604,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" ht="15" customHeight="1" thickBot="1">
       <c r="A3" s="159">
         <v>45911</v>
       </c>
@@ -5661,7 +5667,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15" customHeight="1">
       <c r="A4" s="160">
         <v>45917</v>
       </c>
@@ -5730,7 +5736,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="15" customHeight="1">
       <c r="A5" s="160">
         <v>45926</v>
       </c>
@@ -5788,7 +5794,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15" customHeight="1">
       <c r="A6" s="160">
         <v>45939</v>
       </c>
@@ -5852,7 +5858,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="15" customHeight="1">
       <c r="A7" s="160">
         <v>45946</v>
       </c>
@@ -5909,7 +5915,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="15" customHeight="1">
       <c r="A8" s="160">
         <v>45953</v>
       </c>
@@ -5967,7 +5973,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="15" customHeight="1">
       <c r="A9" s="160">
         <v>45967</v>
       </c>
@@ -6029,7 +6035,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15" customHeight="1">
       <c r="A10" s="160">
         <v>45974</v>
       </c>
@@ -6092,7 +6098,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="15" customHeight="1">
       <c r="A11" s="160">
         <v>45980</v>
       </c>
@@ -6143,7 +6149,7 @@
       <c r="X11" s="35"/>
       <c r="Y11" s="35"/>
     </row>
-    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1">
       <c r="A12" s="160">
         <f>A10+7</f>
         <v>45981</v>
@@ -6196,7 +6202,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25">
       <c r="A13" s="160">
         <v>45986</v>
       </c>
@@ -6232,7 +6238,7 @@
       <c r="M13" s="158"/>
       <c r="N13" s="158"/>
     </row>
-    <row r="14" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="15" customHeight="1">
       <c r="A14" s="160">
         <v>45988</v>
       </c>
@@ -6287,7 +6293,7 @@
       <c r="X14" s="15"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25" ht="15" customHeight="1" thickBot="1">
       <c r="A15" s="161">
         <v>45995</v>
       </c>
@@ -6350,35 +6356,35 @@
       <c r="X15" s="15"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:25" ht="15" customHeight="1" thickBot="1">
       <c r="A16" s="26"/>
       <c r="B16" s="26"/>
       <c r="C16" s="26"/>
       <c r="X16" s="20"/>
       <c r="Y16" s="18"/>
     </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="15" customHeight="1">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
     </row>
-    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="15" customHeight="1">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
     </row>
-    <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="15" customHeight="1">
       <c r="A19" s="26"/>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
     </row>
-    <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:3" ht="15" customHeight="1"/>
+    <row r="21" spans="1:3" ht="15" customHeight="1"/>
+    <row r="22" spans="1:3" ht="15" customHeight="1"/>
+    <row r="23" spans="1:3" ht="15" customHeight="1"/>
+    <row r="24" spans="1:3" ht="15" customHeight="1"/>
+    <row r="25" spans="1:3" ht="15" customHeight="1"/>
+    <row r="26" spans="1:3" ht="15" customHeight="1"/>
   </sheetData>
   <protectedRanges>
     <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A3:E19" name="Range3_1"/>
@@ -6412,7 +6418,7 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1:Y18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -6439,7 +6445,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6450,7 +6456,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" ht="30">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -6527,7 +6533,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15" customHeight="1">
       <c r="A3" s="75">
         <v>46051</v>
       </c>
@@ -6576,7 +6582,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1">
       <c r="A4" s="75">
         <f>A3+12</f>
         <v>46063</v>
@@ -6627,7 +6633,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" ht="18.75" customHeight="1">
       <c r="A5" s="75">
         <f>A4+16</f>
         <v>46079</v>
@@ -6682,7 +6688,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1">
       <c r="A6" s="75">
         <f>A5+14</f>
         <v>46093</v>
@@ -6737,7 +6743,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1">
       <c r="A7" s="75">
         <f>A6+7</f>
         <v>46100</v>
@@ -6791,7 +6797,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" ht="17.25" customHeight="1">
       <c r="A8" s="75">
         <f>A6+14</f>
         <v>46107</v>
@@ -6844,7 +6850,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="18" customHeight="1">
       <c r="A9" s="75">
         <f>A8+7</f>
         <v>46114</v>
@@ -6898,7 +6904,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" ht="15" customHeight="1">
       <c r="A10" s="75">
         <v>46120</v>
       </c>
@@ -6947,7 +6953,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="14.25" customHeight="1">
       <c r="A11" s="75">
         <v>46121</v>
       </c>
@@ -6998,7 +7004,7 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1">
       <c r="A12" s="75">
         <v>46128</v>
       </c>
@@ -7051,7 +7057,7 @@
       <c r="X12" s="15"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" ht="18.75" customHeight="1">
       <c r="A13" s="75">
         <v>46135</v>
       </c>
@@ -7080,7 +7086,7 @@
         <v>376</v>
       </c>
       <c r="J13" s="98" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K13" s="102"/>
       <c r="L13" s="5"/>
@@ -7098,7 +7104,7 @@
       <c r="X13" s="15"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" ht="18.75" customHeight="1">
       <c r="A14" s="75">
         <v>46142</v>
       </c>
@@ -7106,7 +7112,7 @@
         <v>259</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D14" s="27" t="s">
         <v>278</v>
@@ -7115,26 +7121,26 @@
         <v>14</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>431</v>
+        <v>381</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>432</v>
+        <v>382</v>
       </c>
       <c r="J14" s="107" t="s">
-        <v>433</v>
+        <v>383</v>
       </c>
       <c r="K14" s="102" t="s">
-        <v>435</v>
+        <v>384</v>
       </c>
       <c r="L14" s="14"/>
       <c r="M14" s="102" t="s">
-        <v>434</v>
+        <v>385</v>
       </c>
       <c r="N14" s="14"/>
       <c r="O14" s="35"/>
@@ -7149,7 +7155,7 @@
       <c r="X14" s="15"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25" ht="15.75" thickBot="1">
       <c r="A15" s="26">
         <v>46156</v>
       </c>
@@ -7157,7 +7163,7 @@
         <v>190</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D15" t="s">
         <v>278</v>
@@ -7166,34 +7172,34 @@
         <v>16</v>
       </c>
       <c r="F15" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="G15" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="H15" t="s">
         <v>40</v>
       </c>
       <c r="I15" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="J15" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="X15" s="20"/>
       <c r="Y15" s="18"/>
     </row>
-    <row r="16" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" ht="12.75" customHeight="1">
       <c r="A16" s="26"/>
       <c r="B16" s="26"/>
       <c r="C16" s="26"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
@@ -7230,7 +7236,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A33E49C-EC2E-42B7-80E4-DD607C0B7A89}">
   <dimension ref="A1:Y13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -7257,7 +7263,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" ht="15.75" thickBot="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7268,7 +7274,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" ht="30.75" thickBot="1">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -7345,7 +7351,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="15" customHeight="1">
       <c r="A3" s="75">
         <v>46275</v>
       </c>
@@ -7364,19 +7370,19 @@
         <v>1</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="H3" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="I3" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="J3" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="K3" s="73"/>
       <c r="L3" s="40"/>
@@ -7394,7 +7400,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1">
       <c r="A4" s="75">
         <f>A3+14</f>
         <v>46289</v>
@@ -7415,19 +7421,19 @@
         <v>3</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="I4" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="J4" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="K4" s="102"/>
       <c r="L4" s="5"/>
@@ -7445,7 +7451,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25">
       <c r="A5" s="75">
         <f t="shared" ref="A5" si="2">A4+14</f>
         <v>46303</v>
@@ -7466,19 +7472,19 @@
         <v>5</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="I5" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="J5" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="K5" s="102"/>
       <c r="L5" s="5"/>
@@ -7500,7 +7506,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1">
       <c r="A6" s="75">
         <f>A5+14</f>
         <v>46317</v>
@@ -7521,19 +7527,19 @@
         <v>7</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="H6" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="I6" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="J6" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="K6" s="102"/>
       <c r="L6" s="5"/>
@@ -7551,7 +7557,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25">
       <c r="A7" s="75">
         <f>A6+14</f>
         <v>46331</v>
@@ -7572,19 +7578,19 @@
         <v>9</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="I7" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="J7" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="K7" s="102"/>
       <c r="L7" s="5"/>
@@ -7602,7 +7608,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25">
       <c r="A8" s="75">
         <f>A7+14</f>
         <v>46345</v>
@@ -7621,19 +7627,19 @@
         <v>11</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="I8" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="J8" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="K8" s="102"/>
       <c r="L8" s="5"/>
@@ -7651,7 +7657,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" ht="18.75" customHeight="1">
       <c r="A9" s="75">
         <v>46121</v>
       </c>
@@ -7659,7 +7665,7 @@
         <v>190</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D9" s="27" t="s">
         <v>278</v>
@@ -7668,19 +7674,19 @@
         <v>13</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="I9" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="J9" s="98" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="K9" s="102"/>
       <c r="L9" s="5"/>
@@ -7698,24 +7704,24 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" ht="15.75" thickBot="1">
       <c r="A10" s="26"/>
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
       <c r="X10" s="20"/>
       <c r="Y10" s="18"/>
     </row>
-    <row r="11" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" ht="12.75" customHeight="1">
       <c r="A11" s="26"/>
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25">
       <c r="A12" s="26"/>
       <c r="B12" s="26"/>
       <c r="C12" s="26"/>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25">
       <c r="A13" s="26"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
@@ -7737,212 +7743,212 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AEC079F-155A-491D-9189-1418FC903287}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.28515625" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" s="55" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="B2" s="54" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" s="136" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="B3" s="137"/>
       <c r="C3" s="138" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="B4" s="52"/>
       <c r="C4" s="50" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" s="52" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="B5" s="52"/>
       <c r="C5" s="50" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="52" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B6" s="52" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="C6" s="50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" s="52" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="B7" s="52" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="C7" s="50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" s="52" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="C8" s="50" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" s="52" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="B9" s="52"/>
       <c r="C9" s="50"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" s="52" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" s="52" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="B11" s="52" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" s="52" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B12" s="52" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" s="52" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="B13" s="52" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" s="52" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" s="52" t="s">
+        <v>417</v>
+      </c>
+      <c r="B15" s="52" t="s">
+        <v>418</v>
+      </c>
+      <c r="C15" s="50" t="s">
         <v>410</v>
       </c>
-      <c r="B15" s="52" t="s">
-        <v>411</v>
-      </c>
-      <c r="C15" s="50" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" s="137" t="s">
         <v>321</v>
       </c>
       <c r="B16" s="137" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="C16" s="139" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" s="137" t="s">
         <v>346</v>
       </c>
       <c r="B17" s="137" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="C17" s="139" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" s="52" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="C18" s="50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" s="53" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="B19" s="53" t="s">
         <v>230</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="B20" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
     </row>
   </sheetData>
@@ -7958,24 +7964,24 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD19DE5-C22F-4D41-B540-76D70438E18B}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="6" max="6" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1">
       <c r="A1" s="135" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="131" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="C1" s="130" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="169">
         <v>46051</v>
       </c>
@@ -7983,14 +7989,14 @@
         <v>1</v>
       </c>
       <c r="C2" s="170" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="F2" s="75"/>
       <c r="G2" s="77"/>
       <c r="H2" s="29"/>
       <c r="I2" s="55"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9">
       <c r="A3" s="171">
         <f>A2+7</f>
         <v>46058</v>
@@ -8000,14 +8006,14 @@
         <v>2</v>
       </c>
       <c r="C3" s="170" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="F3" s="75"/>
       <c r="G3" s="2"/>
       <c r="H3" s="26"/>
       <c r="I3" s="27"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9">
       <c r="A4" s="171">
         <f t="shared" ref="A4:A12" si="0">A3+7</f>
         <v>46065</v>
@@ -8017,14 +8023,14 @@
         <v>3</v>
       </c>
       <c r="C4" s="170" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="F4" s="75"/>
       <c r="G4" s="2"/>
       <c r="H4" s="26"/>
       <c r="I4" s="27"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9">
       <c r="A5" s="171">
         <f t="shared" si="0"/>
         <v>46072</v>
@@ -8034,14 +8040,14 @@
         <v>4</v>
       </c>
       <c r="C5" s="170" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="F5" s="75"/>
       <c r="G5" s="2"/>
       <c r="H5" s="26"/>
       <c r="I5" s="27"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9">
       <c r="A6" s="133">
         <f t="shared" si="0"/>
         <v>46079</v>
@@ -8051,14 +8057,14 @@
         <v>5</v>
       </c>
       <c r="C6" s="134" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="F6" s="75"/>
       <c r="G6" s="2"/>
       <c r="H6" s="26"/>
       <c r="I6" s="27"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="A7" s="133">
         <f t="shared" si="0"/>
         <v>46086</v>
@@ -8068,14 +8074,14 @@
         <v>6</v>
       </c>
       <c r="C7" s="134" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="F7" s="75"/>
       <c r="G7" s="2"/>
       <c r="H7" s="26"/>
       <c r="I7" s="27"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9">
       <c r="A8" s="133">
         <f t="shared" si="0"/>
         <v>46093</v>
@@ -8085,14 +8091,14 @@
         <v>7</v>
       </c>
       <c r="C8" s="134" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="F8" s="75"/>
       <c r="G8" s="2"/>
       <c r="H8" s="26"/>
       <c r="I8" s="27"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9">
       <c r="A9" s="133">
         <f t="shared" si="0"/>
         <v>46100</v>
@@ -8102,14 +8108,14 @@
         <v>8</v>
       </c>
       <c r="C9" s="134" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="F9" s="75"/>
       <c r="G9" s="2"/>
       <c r="H9" s="26"/>
       <c r="I9" s="27"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9">
       <c r="A10" s="133">
         <f t="shared" si="0"/>
         <v>46107</v>
@@ -8119,14 +8125,14 @@
         <v>9</v>
       </c>
       <c r="C10" s="134" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="F10" s="75"/>
       <c r="G10" s="2"/>
       <c r="H10" s="26"/>
       <c r="I10" s="27"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9">
       <c r="A11" s="133">
         <f t="shared" si="0"/>
         <v>46114</v>
@@ -8136,10 +8142,10 @@
         <v>10</v>
       </c>
       <c r="C11" s="134" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" s="133">
         <f t="shared" si="0"/>
         <v>46121</v>
@@ -8149,10 +8155,10 @@
         <v>11</v>
       </c>
       <c r="C12" s="134" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
       <c r="A13" s="133">
         <f t="shared" ref="A13:A14" si="3">A12+7</f>
         <v>46128</v>
@@ -8162,10 +8168,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="134" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
       <c r="A14" s="133">
         <f t="shared" si="3"/>
         <v>46135</v>
@@ -8175,15 +8181,15 @@
         <v>13</v>
       </c>
       <c r="C14" s="134" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
       <c r="A15" s="133"/>
       <c r="B15" s="134"/>
       <c r="C15" s="134"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9">
       <c r="G16" s="26"/>
     </row>
   </sheetData>
@@ -8210,7 +8216,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2BB5C5F-5790-4A91-A6E8-8841719DA1FC}">
   <dimension ref="A2:I20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.42578125" customWidth="1"/>
     <col min="2" max="2" width="9.140625" customWidth="1"/>
@@ -8222,17 +8228,17 @@
     <col min="9" max="9" width="64.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" ht="23.25" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="23.25">
       <c r="A2" s="91" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="18.75">
       <c r="A3" s="79" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="37.5">
       <c r="A5" s="80" t="s">
         <v>3</v>
       </c>
@@ -8255,13 +8261,13 @@
         <v>9</v>
       </c>
       <c r="H5" s="82" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="I5" s="81" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="18.75">
       <c r="A6" s="92">
         <v>45694</v>
       </c>
@@ -8285,10 +8291,10 @@
       </c>
       <c r="H6" s="85"/>
       <c r="I6" s="84" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="18.75">
       <c r="A7" s="83">
         <v>45708</v>
       </c>
@@ -8317,7 +8323,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="18.75">
       <c r="A8" s="83">
         <v>45722</v>
       </c>
@@ -8344,7 +8350,7 @@
       </c>
       <c r="I8" s="86"/>
     </row>
-    <row r="9" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="18.75">
       <c r="A9" s="83">
         <v>45735</v>
       </c>
@@ -8355,7 +8361,7 @@
         <v>198</v>
       </c>
       <c r="D9" s="94" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="E9" s="94">
         <v>8</v>
@@ -8370,10 +8376,10 @@
         <v>206</v>
       </c>
       <c r="I9" s="86" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="18.75">
       <c r="A10" s="83">
         <v>45744</v>
       </c>
@@ -8400,7 +8406,7 @@
       </c>
       <c r="I10" s="86"/>
     </row>
-    <row r="11" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="18.75">
       <c r="A11" s="83">
         <v>45750</v>
       </c>
@@ -8417,17 +8423,17 @@
         <v>10</v>
       </c>
       <c r="F11" s="87" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="G11" s="87" t="s">
         <v>68</v>
       </c>
       <c r="H11" s="87"/>
       <c r="I11" s="86" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="18.75">
       <c r="A12" s="83">
         <v>45758</v>
       </c>
@@ -8453,10 +8459,10 @@
         <v>31</v>
       </c>
       <c r="I12" s="86" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="18.75">
       <c r="A13" s="83">
         <v>45764</v>
       </c>
@@ -8473,13 +8479,13 @@
         <v>12</v>
       </c>
       <c r="F13" s="87" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="G13" s="87"/>
       <c r="H13" s="87"/>
       <c r="I13" s="86"/>
     </row>
-    <row r="14" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="18.75">
       <c r="A14" s="88">
         <v>45771</v>
       </c>
@@ -8496,7 +8502,7 @@
         <v>13</v>
       </c>
       <c r="F14" s="90" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="G14" s="90" t="s">
         <v>77</v>
@@ -8508,7 +8514,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="20" spans="8:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="20" spans="8:8" ht="18.75">
       <c r="H20" s="79"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change time of NK's talk
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="416" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8ABB13C-981A-4743-ABF0-CA69466D205E}"/>
+  <xr:revisionPtr revIDLastSave="420" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C7A8884-F82B-402B-8234-55823CB0D8A3}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1268,6 +1268,9 @@
     <t>https://ffaucher.gitlab.io/cv/</t>
   </si>
   <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
     <t>Alan Demlow</t>
   </si>
   <si>
@@ -1410,9 +1413,6 @@
   </si>
   <si>
     <t>Deptartmental contact</t>
-  </si>
-  <si>
-    <t>Wednesday</t>
   </si>
   <si>
     <t>Robery Garvey</t>
@@ -7157,7 +7157,7 @@
     </row>
     <row r="15" spans="1:25" ht="15.75" thickBot="1">
       <c r="A15" s="26">
-        <v>46156</v>
+        <v>46155</v>
       </c>
       <c r="B15" s="26" t="s">
         <v>190</v>
@@ -7166,25 +7166,25 @@
         <v>378</v>
       </c>
       <c r="D15" t="s">
-        <v>278</v>
+        <v>386</v>
       </c>
       <c r="E15">
         <v>16</v>
       </c>
       <c r="F15" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G15" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="H15" t="s">
         <v>40</v>
       </c>
       <c r="I15" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J15" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="X15" s="20"/>
       <c r="Y15" s="18"/>
@@ -7370,19 +7370,19 @@
         <v>1</v>
       </c>
       <c r="F3" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="G3" s="14" t="s">
-        <v>388</v>
-      </c>
       <c r="H3" s="14" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I3" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J3" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K3" s="73"/>
       <c r="L3" s="40"/>
@@ -7421,19 +7421,19 @@
         <v>3</v>
       </c>
       <c r="F4" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="G4" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="G4" s="14" t="s">
-        <v>388</v>
-      </c>
       <c r="H4" s="5" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I4" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J4" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K4" s="102"/>
       <c r="L4" s="5"/>
@@ -7472,19 +7472,19 @@
         <v>5</v>
       </c>
       <c r="F5" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="G5" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="G5" s="14" t="s">
-        <v>388</v>
-      </c>
       <c r="H5" s="14" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I5" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J5" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K5" s="102"/>
       <c r="L5" s="5"/>
@@ -7527,19 +7527,19 @@
         <v>7</v>
       </c>
       <c r="F6" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="G6" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="G6" s="14" t="s">
-        <v>388</v>
-      </c>
       <c r="H6" s="14" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I6" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J6" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K6" s="102"/>
       <c r="L6" s="5"/>
@@ -7578,19 +7578,19 @@
         <v>9</v>
       </c>
       <c r="F7" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="G7" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="G7" s="14" t="s">
-        <v>388</v>
-      </c>
       <c r="H7" s="14" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I7" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J7" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K7" s="102"/>
       <c r="L7" s="5"/>
@@ -7627,19 +7627,19 @@
         <v>11</v>
       </c>
       <c r="F8" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="G8" s="14" t="s">
-        <v>388</v>
-      </c>
       <c r="H8" s="14" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I8" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J8" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K8" s="102"/>
       <c r="L8" s="5"/>
@@ -7674,19 +7674,19 @@
         <v>13</v>
       </c>
       <c r="F9" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="G9" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="G9" s="14" t="s">
-        <v>388</v>
-      </c>
       <c r="H9" s="14" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I9" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J9" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K9" s="102"/>
       <c r="L9" s="5"/>
@@ -7752,23 +7752,23 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="55" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B2" s="54" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="136" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B3" s="137"/>
       <c r="C3" s="138" t="s">
@@ -7777,7 +7777,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="5" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B4" s="52"/>
       <c r="C4" s="50" t="s">
@@ -7786,19 +7786,19 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="52" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B5" s="52"/>
       <c r="C5" s="50" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="52" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B6" s="52" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C6" s="50" t="s">
         <v>87</v>
@@ -7806,10 +7806,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="52" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B7" s="52" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C7" s="50" t="s">
         <v>87</v>
@@ -7817,10 +7817,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="52" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B8" s="52" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C8" s="50" t="s">
         <v>101</v>
@@ -7828,75 +7828,75 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="52" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B9" s="52"/>
       <c r="C9" s="50"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="52" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B10" s="52" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="52" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B11" s="52" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="52" t="s">
+        <v>412</v>
+      </c>
+      <c r="B12" s="52" t="s">
+        <v>413</v>
+      </c>
+      <c r="C12" s="50" t="s">
         <v>411</v>
-      </c>
-      <c r="B12" s="52" t="s">
-        <v>412</v>
-      </c>
-      <c r="C12" s="50" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="52" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B13" s="52" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="52" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B14" s="52" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="52" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B15" s="52" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -7904,10 +7904,10 @@
         <v>321</v>
       </c>
       <c r="B16" s="137" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C16" s="139" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7915,18 +7915,18 @@
         <v>346</v>
       </c>
       <c r="B17" s="137" t="s">
+        <v>422</v>
+      </c>
+      <c r="C17" s="139" t="s">
         <v>421</v>
-      </c>
-      <c r="C17" s="139" t="s">
-        <v>420</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="52" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B18" s="52" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C18" s="50" t="s">
         <v>87</v>
@@ -7934,21 +7934,21 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="53" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B19" s="53" t="s">
         <v>230</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B20" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
   </sheetData>
@@ -7975,10 +7975,10 @@
         <v>3</v>
       </c>
       <c r="B1" s="131" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C1" s="130" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -7989,7 +7989,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="170" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F2" s="75"/>
       <c r="G2" s="77"/>
@@ -8006,7 +8006,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="170" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F3" s="75"/>
       <c r="G3" s="2"/>
@@ -8023,7 +8023,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="170" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F4" s="75"/>
       <c r="G4" s="2"/>
@@ -8040,7 +8040,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="170" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F5" s="75"/>
       <c r="G5" s="2"/>
@@ -8057,7 +8057,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="134" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F6" s="75"/>
       <c r="G6" s="2"/>
@@ -8074,7 +8074,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="134" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F7" s="75"/>
       <c r="G7" s="2"/>
@@ -8091,7 +8091,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="134" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F8" s="75"/>
       <c r="G8" s="2"/>
@@ -8108,7 +8108,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="134" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F9" s="75"/>
       <c r="G9" s="2"/>
@@ -8125,7 +8125,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="134" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F10" s="75"/>
       <c r="G10" s="2"/>
@@ -8142,7 +8142,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="134" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -8155,7 +8155,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="134" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -8168,7 +8168,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="134" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -8181,7 +8181,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="134" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -8230,12 +8230,12 @@
   <sheetData>
     <row r="2" spans="1:9" ht="23.25">
       <c r="A2" s="91" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="18.75">
       <c r="A3" s="79" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="37.5">
@@ -8261,7 +8261,7 @@
         <v>9</v>
       </c>
       <c r="H5" s="82" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="I5" s="81" t="s">
         <v>11</v>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="H6" s="85"/>
       <c r="I6" s="84" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="18.75">
@@ -8361,7 +8361,7 @@
         <v>198</v>
       </c>
       <c r="D9" s="94" t="s">
-        <v>434</v>
+        <v>386</v>
       </c>
       <c r="E9" s="94">
         <v>8</v>
@@ -8376,7 +8376,7 @@
         <v>206</v>
       </c>
       <c r="I9" s="86" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="18.75">
@@ -8430,7 +8430,7 @@
       </c>
       <c r="H11" s="87"/>
       <c r="I11" s="86" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="18.75">
@@ -8459,7 +8459,7 @@
         <v>31</v>
       </c>
       <c r="I12" s="86" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="18.75">

</xml_diff>

<commit_message>
updated PMC spkeakers name
</commit_message>
<xml_diff>
--- a/data/MACSI seminar series.xlsx
+++ b/data/MACSI seminar series.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ulcampus-my.sharepoint.com/personal/david_osullivan_ul_ie/Documents/Academic_work/_Misc/MACSI Seminars/macsi-seminars.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="440" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BACF11D6-FBAB-4DAF-90D2-E3CDAB0DBA6A}"/>
+  <xr:revisionPtr revIDLastSave="444" documentId="13_ncr:1_{12BE53B5-C8C7-44FE-8280-19C653D9122E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B65A9E4-15AD-47F3-AF5C-6B2EA0E64C24}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4410" yWindow="4185" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AY2023-2024 Sem 2" sheetId="3" state="hidden" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="443">
   <si>
     <t>Fill in as much of the green boxes as possible. Ideally, this would be before you have finished your visitors travel dates (just to avoid double booking).</t>
   </si>
@@ -1287,15 +1287,15 @@
     <t>June</t>
   </si>
   <si>
+    <t>TBC</t>
+  </si>
+  <si>
     <t>Warwick University</t>
   </si>
   <si>
     <t>Open</t>
   </si>
   <si>
-    <t>TBC</t>
-  </si>
-  <si>
     <t>This is a just a place for those who are interested but that dont have a specific date in mind. (Ideally, a couple of these are people that we could invite with relatively short notice to fill missing slots.)</t>
   </si>
   <si>
@@ -1435,6 +1435,9 @@
   </si>
   <si>
     <t>Leornard Henckel</t>
+  </si>
+  <si>
+    <t>Martine Barons</t>
   </si>
 </sst>
 </file>
@@ -1444,7 +1447,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2302,9 +2305,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2342,7 +2345,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2448,7 +2451,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2590,7 +2593,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2599,7 +2602,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7958562-D4BB-4776-9668-682A6F2E2AD0}">
   <dimension ref="A1:Y20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="11.140625" customWidth="1"/>
@@ -2624,7 +2627,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2635,7 +2638,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30">
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -2712,7 +2715,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="13.5" customHeight="1">
+    <row r="3" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45317</v>
       </c>
@@ -2779,7 +2782,7 @@
       <c r="X3" s="13"/>
       <c r="Y3" s="13"/>
     </row>
-    <row r="4" spans="1:25" ht="13.5" customHeight="1">
+    <row r="4" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45323</v>
       </c>
@@ -2842,7 +2845,7 @@
       <c r="X4" s="13"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45324</v>
       </c>
@@ -2903,7 +2906,7 @@
       <c r="X5" s="13"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="12.75" customHeight="1">
+    <row r="6" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45331</v>
       </c>
@@ -2970,7 +2973,7 @@
       <c r="X6" s="13"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45338</v>
       </c>
@@ -3039,7 +3042,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1">
+    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45345</v>
       </c>
@@ -3106,7 +3109,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="16.5" customHeight="1">
+    <row r="9" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45359</v>
       </c>
@@ -3159,7 +3162,7 @@
       <c r="X9" s="13"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45366</v>
       </c>
@@ -3228,7 +3231,7 @@
       <c r="X10" s="13"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1">
+    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>45379</v>
       </c>
@@ -3289,7 +3292,7 @@
       <c r="X11" s="13"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="13.5" customHeight="1">
+    <row r="12" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>45386</v>
       </c>
@@ -3352,7 +3355,7 @@
       <c r="X12" s="13"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="16.5" customHeight="1">
+    <row r="13" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>45387</v>
       </c>
@@ -3421,7 +3424,7 @@
       <c r="X13" s="13"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>45394</v>
       </c>
@@ -3482,7 +3485,7 @@
       <c r="X14" s="13"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="17.25" customHeight="1">
+    <row r="15" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>45398</v>
       </c>
@@ -3551,7 +3554,7 @@
       <c r="X15" s="13"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>45401</v>
       </c>
@@ -3614,7 +3617,7 @@
       <c r="X16" s="18"/>
       <c r="Y16" s="18"/>
     </row>
-    <row r="17" spans="1:25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>45421</v>
       </c>
@@ -3685,7 +3688,7 @@
       <c r="X17" s="18"/>
       <c r="Y17" s="18"/>
     </row>
-    <row r="18" spans="1:25">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="26">
         <v>45474</v>
       </c>
@@ -3736,7 +3739,7 @@
       <c r="X18" s="18"/>
       <c r="Y18" s="18"/>
     </row>
-    <row r="19" spans="1:25" ht="17.25" customHeight="1" thickBot="1">
+    <row r="19" spans="1:25" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="26">
         <v>45505</v>
       </c>
@@ -3787,7 +3790,7 @@
       <c r="X19" s="18"/>
       <c r="Y19" s="18"/>
     </row>
-    <row r="20" spans="1:25">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="26"/>
       <c r="B20" s="26"/>
       <c r="C20" s="26"/>
@@ -3829,7 +3832,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y44"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="11.140625" customWidth="1"/>
@@ -3854,7 +3857,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3865,7 +3868,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30.75" thickBot="1">
+    <row r="2" spans="1:25" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="145" t="s">
         <v>3</v>
       </c>
@@ -3942,7 +3945,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45548</v>
       </c>
@@ -4007,7 +4010,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15" customHeight="1">
+    <row r="4" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45555</v>
       </c>
@@ -4056,7 +4059,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="15" customHeight="1">
+    <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45562</v>
       </c>
@@ -4105,7 +4108,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15" customHeight="1">
+    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45576</v>
       </c>
@@ -4154,7 +4157,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15" customHeight="1">
+    <row r="7" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45583</v>
       </c>
@@ -4203,7 +4206,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1">
+    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45596</v>
       </c>
@@ -4252,7 +4255,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15" customHeight="1">
+    <row r="9" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45604</v>
       </c>
@@ -4301,7 +4304,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1">
+    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45611</v>
       </c>
@@ -4350,7 +4353,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1">
+    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>45625</v>
       </c>
@@ -4399,7 +4402,7 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="15" customHeight="1" thickBot="1">
+    <row r="12" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>45632</v>
       </c>
@@ -4456,20 +4459,20 @@
       <c r="X12" s="20"/>
       <c r="Y12" s="18"/>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="26"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
       <c r="D13" s="26"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="26"/>
       <c r="B14" s="26"/>
       <c r="C14" s="26"/>
       <c r="D14" s="26"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -4481,59 +4484,59 @@
       <c r="I29" s="61"/>
       <c r="J29" s="61"/>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="60"/>
       <c r="B31" s="60"/>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="60"/>
       <c r="B32" s="60"/>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="60"/>
       <c r="B33" s="60"/>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="60"/>
       <c r="B34" s="60"/>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="60"/>
       <c r="B35" s="60"/>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="60"/>
       <c r="B36" s="60"/>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="60"/>
       <c r="B37" s="60"/>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="60"/>
       <c r="B38" s="60"/>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="60"/>
       <c r="B39" s="60"/>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="60"/>
       <c r="B40" s="60"/>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="60"/>
       <c r="B41" s="60"/>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="60"/>
       <c r="B42" s="60"/>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="60"/>
       <c r="B43" s="60"/>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="60"/>
       <c r="B44" s="60"/>
     </row>
@@ -4562,7 +4565,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12299A9A-6C0C-4F92-957E-FBFCB6211744}">
   <dimension ref="A1:Y45"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="5.85546875" bestFit="1" customWidth="1"/>
@@ -4590,7 +4593,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4601,7 +4604,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="27.75" customHeight="1" thickBot="1">
+    <row r="2" spans="1:25" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -4678,7 +4681,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>45694</v>
       </c>
@@ -4730,7 +4733,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="14.25" customHeight="1">
+    <row r="4" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>45708</v>
       </c>
@@ -4788,7 +4791,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="14.25" customHeight="1">
+    <row r="5" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>45722</v>
       </c>
@@ -4844,7 +4847,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="16.5" customHeight="1">
+    <row r="6" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>45735</v>
       </c>
@@ -4900,7 +4903,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="18" customHeight="1">
+    <row r="7" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>45750</v>
       </c>
@@ -4954,7 +4957,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="16.5" customHeight="1">
+    <row r="8" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>45751</v>
       </c>
@@ -5013,7 +5016,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15.75" customHeight="1">
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>45757</v>
       </c>
@@ -5075,7 +5078,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" customHeight="1">
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>45758</v>
       </c>
@@ -5129,7 +5132,7 @@
       <c r="X10" s="20"/>
       <c r="Y10" s="18"/>
     </row>
-    <row r="11" spans="1:25" ht="15.75" customHeight="1">
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>45764</v>
       </c>
@@ -5189,7 +5192,7 @@
       <c r="X11" s="35"/>
       <c r="Y11" s="35"/>
     </row>
-    <row r="12" spans="1:25" ht="15.75" customHeight="1">
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>45771</v>
       </c>
@@ -5250,7 +5253,7 @@
       <c r="X12" s="35"/>
       <c r="Y12" s="35"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75" customHeight="1">
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>45785</v>
       </c>
@@ -5303,7 +5306,7 @@
       <c r="X13" s="35"/>
       <c r="Y13" s="35"/>
     </row>
-    <row r="14" spans="1:25" ht="15.75" customHeight="1">
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>45799</v>
       </c>
@@ -5349,7 +5352,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.75" customHeight="1">
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>45805</v>
       </c>
@@ -5383,101 +5386,101 @@
         <v>250</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15.75" customHeight="1">
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="75"/>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="26"/>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="26"/>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="26"/>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="75"/>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="26"/>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="75"/>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="26"/>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="26"/>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="26"/>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="26"/>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="26"/>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="26"/>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B31" s="60"/>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="60"/>
       <c r="B32" s="60"/>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="60"/>
       <c r="B33" s="60"/>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="60"/>
       <c r="B34" s="60"/>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="60"/>
       <c r="B35" s="60"/>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="60"/>
       <c r="B36" s="60"/>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="60"/>
       <c r="B37" s="60"/>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="60"/>
       <c r="B38" s="60"/>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="60"/>
       <c r="B39" s="60"/>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="60"/>
       <c r="B40" s="60"/>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="60"/>
       <c r="B41" s="60"/>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="60"/>
       <c r="B42" s="60"/>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="60"/>
       <c r="B43" s="60"/>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="60"/>
       <c r="B44" s="60"/>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="60"/>
     </row>
   </sheetData>
@@ -5502,7 +5505,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{243C2AD8-98F5-4435-96A3-1C2CAB922825}">
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
@@ -5529,7 +5532,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5540,7 +5543,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30">
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="78" t="s">
         <v>3</v>
       </c>
@@ -5617,7 +5620,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1" thickBot="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="159">
         <v>45911</v>
       </c>
@@ -5680,7 +5683,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15" customHeight="1">
+    <row r="4" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="160">
         <v>45917</v>
       </c>
@@ -5749,7 +5752,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="15" customHeight="1">
+    <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="160">
         <v>45926</v>
       </c>
@@ -5807,7 +5810,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15" customHeight="1">
+    <row r="6" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="160">
         <v>45939</v>
       </c>
@@ -5871,7 +5874,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15" customHeight="1">
+    <row r="7" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="160">
         <v>45946</v>
       </c>
@@ -5928,7 +5931,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="15" customHeight="1">
+    <row r="8" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="160">
         <v>45953</v>
       </c>
@@ -5986,7 +5989,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="15" customHeight="1">
+    <row r="9" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="160">
         <v>45967</v>
       </c>
@@ -6048,7 +6051,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1">
+    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="160">
         <v>45974</v>
       </c>
@@ -6111,7 +6114,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="15" customHeight="1">
+    <row r="11" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="160">
         <v>45980</v>
       </c>
@@ -6162,7 +6165,7 @@
       <c r="X11" s="35"/>
       <c r="Y11" s="35"/>
     </row>
-    <row r="12" spans="1:25" ht="16.5" customHeight="1">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="160">
         <f>A10+7</f>
         <v>45981</v>
@@ -6215,7 +6218,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="160">
         <v>45986</v>
       </c>
@@ -6251,7 +6254,7 @@
       <c r="M13" s="158"/>
       <c r="N13" s="158"/>
     </row>
-    <row r="14" spans="1:25" ht="15" customHeight="1">
+    <row r="14" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="160">
         <v>45988</v>
       </c>
@@ -6306,7 +6309,7 @@
       <c r="X14" s="15"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="15" customHeight="1" thickBot="1">
+    <row r="15" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="161">
         <v>45995</v>
       </c>
@@ -6369,35 +6372,35 @@
       <c r="X15" s="15"/>
       <c r="Y15" s="13"/>
     </row>
-    <row r="16" spans="1:25" ht="15" customHeight="1" thickBot="1">
+    <row r="16" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="26"/>
       <c r="B16" s="26"/>
       <c r="C16" s="26"/>
       <c r="X16" s="20"/>
       <c r="Y16" s="18"/>
     </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1">
+    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
     </row>
-    <row r="18" spans="1:3" ht="15" customHeight="1">
+    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
     </row>
-    <row r="19" spans="1:3" ht="15" customHeight="1">
+    <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="26"/>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
     </row>
-    <row r="20" spans="1:3" ht="15" customHeight="1"/>
-    <row r="21" spans="1:3" ht="15" customHeight="1"/>
-    <row r="22" spans="1:3" ht="15" customHeight="1"/>
-    <row r="23" spans="1:3" ht="15" customHeight="1"/>
-    <row r="24" spans="1:3" ht="15" customHeight="1"/>
-    <row r="25" spans="1:3" ht="15" customHeight="1"/>
-    <row r="26" spans="1:3" ht="15" customHeight="1"/>
+    <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <protectedRanges>
     <protectedRange algorithmName="SHA-512" hashValue="pQyTzP/d7t5ThMimBt5mu8gGozgAm1OwF6BMILsn5/kmtZ5mZf81NMi09wwU8mvtItxf0EVNWa6V4MCa0DKeSQ==" saltValue="NzZBiAQ1yFjat+SeIqh2Uw==" spinCount="100000" sqref="A3:E19" name="Range3_1"/>
@@ -6431,7 +6434,7 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1:Y18"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -6458,7 +6461,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6469,7 +6472,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30">
+    <row r="2" spans="1:25" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -6546,7 +6549,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="75">
         <v>46051</v>
       </c>
@@ -6595,7 +6598,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="75">
         <f>A3+12</f>
         <v>46063</v>
@@ -6646,7 +6649,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25" ht="18.75" customHeight="1">
+    <row r="5" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="75">
         <f>A4+16</f>
         <v>46079</v>
@@ -6701,7 +6704,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="75">
         <f>A5+14</f>
         <v>46093</v>
@@ -6756,7 +6759,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25" ht="15.75" customHeight="1">
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="75">
         <f>A6+7</f>
         <v>46100</v>
@@ -6810,7 +6813,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25" ht="17.25" customHeight="1">
+    <row r="8" spans="1:25" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="75">
         <f>A6+14</f>
         <v>46107</v>
@@ -6863,7 +6866,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="18" customHeight="1">
+    <row r="9" spans="1:25" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="75">
         <f>A8+7</f>
         <v>46114</v>
@@ -6917,7 +6920,7 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15" customHeight="1">
+    <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="75">
         <v>46120</v>
       </c>
@@ -6966,7 +6969,7 @@
       <c r="X10" s="15"/>
       <c r="Y10" s="13"/>
     </row>
-    <row r="11" spans="1:25" ht="14.25" customHeight="1">
+    <row r="11" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="75">
         <v>46121</v>
       </c>
@@ -7017,7 +7020,7 @@
       <c r="X11" s="15"/>
       <c r="Y11" s="13"/>
     </row>
-    <row r="12" spans="1:25" ht="16.5" customHeight="1">
+    <row r="12" spans="1:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="75">
         <v>46128</v>
       </c>
@@ -7070,7 +7073,7 @@
       <c r="X12" s="15"/>
       <c r="Y12" s="13"/>
     </row>
-    <row r="13" spans="1:25" ht="18.75" customHeight="1">
+    <row r="13" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="75">
         <v>46135</v>
       </c>
@@ -7117,7 +7120,7 @@
       <c r="X13" s="15"/>
       <c r="Y13" s="13"/>
     </row>
-    <row r="14" spans="1:25" ht="18.75" customHeight="1">
+    <row r="14" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="75">
         <v>46142</v>
       </c>
@@ -7168,7 +7171,7 @@
       <c r="X14" s="15"/>
       <c r="Y14" s="13"/>
     </row>
-    <row r="15" spans="1:25" ht="20.25" customHeight="1">
+    <row r="15" spans="1:25" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26">
         <v>46155</v>
       </c>
@@ -7202,7 +7205,7 @@
       <c r="X15" s="20"/>
       <c r="Y15" s="18"/>
     </row>
-    <row r="16" spans="1:25" ht="12.75" customHeight="1">
+    <row r="16" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="26">
         <v>46175</v>
       </c>
@@ -7218,19 +7221,28 @@
       <c r="E16">
         <v>19</v>
       </c>
+      <c r="F16" t="s">
+        <v>442</v>
+      </c>
       <c r="G16" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="H16" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
+      <c r="I16" t="s">
+        <v>392</v>
+      </c>
+      <c r="J16" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="26"/>
       <c r="B17" s="26"/>
       <c r="C17" s="26"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="26"/>
       <c r="B18" s="26"/>
       <c r="C18" s="26"/>
@@ -7267,7 +7279,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A33E49C-EC2E-42B7-80E4-DD607C0B7A89}">
   <dimension ref="A1:Y13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -7294,7 +7306,7 @@
     <col min="25" max="25" width="37.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="15.75" thickBot="1">
+    <row r="1" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7305,7 +7317,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30.75" thickBot="1">
+    <row r="2" spans="1:25" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="64" t="s">
         <v>3</v>
       </c>
@@ -7382,7 +7394,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15" customHeight="1">
+    <row r="3" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="75">
         <v>46275</v>
       </c>
@@ -7401,19 +7413,19 @@
         <v>1</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="H3" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="I3" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="J3" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="K3" s="73"/>
       <c r="L3" s="40"/>
@@ -7431,7 +7443,7 @@
       <c r="X3" s="46"/>
       <c r="Y3" s="44"/>
     </row>
-    <row r="4" spans="1:25" ht="15.75" customHeight="1">
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="75">
         <f>A3+14</f>
         <v>46289</v>
@@ -7452,19 +7464,19 @@
         <v>3</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="I4" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="J4" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="K4" s="102"/>
       <c r="L4" s="5"/>
@@ -7482,7 +7494,7 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="13"/>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="75">
         <f t="shared" ref="A5" si="2">A4+14</f>
         <v>46303</v>
@@ -7503,19 +7515,19 @@
         <v>5</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="I5" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="J5" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="K5" s="102"/>
       <c r="L5" s="5"/>
@@ -7537,7 +7549,7 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="13"/>
     </row>
-    <row r="6" spans="1:25" ht="15.75" customHeight="1">
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="75">
         <f>A5+14</f>
         <v>46317</v>
@@ -7558,19 +7570,19 @@
         <v>7</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="H6" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="I6" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="J6" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="K6" s="102"/>
       <c r="L6" s="5"/>
@@ -7588,7 +7600,7 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="13"/>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="75">
         <f>A6+14</f>
         <v>46331</v>
@@ -7609,19 +7621,19 @@
         <v>9</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="I7" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="J7" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="K7" s="102"/>
       <c r="L7" s="5"/>
@@ -7639,7 +7651,7 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="13"/>
     </row>
-    <row r="8" spans="1:25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="75">
         <f>A7+14</f>
         <v>46345</v>
@@ -7658,19 +7670,19 @@
         <v>11</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="I8" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="J8" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="K8" s="102"/>
       <c r="L8" s="5"/>
@@ -7688,7 +7700,7 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="13"/>
     </row>
-    <row r="9" spans="1:25" ht="18.75" customHeight="1">
+    <row r="9" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="75">
         <v>46121</v>
       </c>
@@ -7705,19 +7717,19 @@
         <v>13</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="I9" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="J9" s="98" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="K9" s="102"/>
       <c r="L9" s="5"/>
@@ -7735,24 +7747,24 @@
       <c r="X9" s="15"/>
       <c r="Y9" s="13"/>
     </row>
-    <row r="10" spans="1:25" ht="15.75" thickBot="1">
+    <row r="10" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="26"/>
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
       <c r="X10" s="20"/>
       <c r="Y10" s="18"/>
     </row>
-    <row r="11" spans="1:25" ht="12.75" customHeight="1">
+    <row r="11" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="26"/>
       <c r="B11" s="26"/>
       <c r="C11" s="26"/>
     </row>
-    <row r="12" spans="1:25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="26"/>
       <c r="B12" s="26"/>
       <c r="C12" s="26"/>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="26"/>
       <c r="B13" s="26"/>
       <c r="C13" s="26"/>
@@ -7774,19 +7786,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AEC079F-155A-491D-9189-1418FC903287}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.28515625" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="55" t="s">
         <v>396</v>
       </c>
@@ -7797,7 +7809,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="136" t="s">
         <v>399</v>
       </c>
@@ -7806,7 +7818,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>400</v>
       </c>
@@ -7815,7 +7827,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="52" t="s">
         <v>401</v>
       </c>
@@ -7824,7 +7836,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="52" t="s">
         <v>403</v>
       </c>
@@ -7835,7 +7847,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="52" t="s">
         <v>405</v>
       </c>
@@ -7846,7 +7858,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="52" t="s">
         <v>407</v>
       </c>
@@ -7857,14 +7869,14 @@
         <v>101</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
         <v>409</v>
       </c>
       <c r="B9" s="52"/>
       <c r="C9" s="50"/>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="52" t="s">
         <v>410</v>
       </c>
@@ -7875,7 +7887,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="52" t="s">
         <v>413</v>
       </c>
@@ -7886,7 +7898,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="52" t="s">
         <v>416</v>
       </c>
@@ -7897,7 +7909,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="52" t="s">
         <v>418</v>
       </c>
@@ -7908,7 +7920,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="52" t="s">
         <v>420</v>
       </c>
@@ -7919,7 +7931,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="52" t="s">
         <v>422</v>
       </c>
@@ -7930,7 +7942,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="137" t="s">
         <v>321</v>
       </c>
@@ -7941,7 +7953,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="137" t="s">
         <v>346</v>
       </c>
@@ -7952,7 +7964,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="52" t="s">
         <v>427</v>
       </c>
@@ -7963,7 +7975,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="53" t="s">
         <v>428</v>
       </c>
@@ -7974,7 +7986,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>430</v>
       </c>
@@ -7995,13 +8007,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD19DE5-C22F-4D41-B540-76D70438E18B}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="6" max="6" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="135" t="s">
         <v>3</v>
       </c>
@@ -8012,7 +8024,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="169">
         <v>46051</v>
       </c>
@@ -8027,7 +8039,7 @@
       <c r="H2" s="29"/>
       <c r="I2" s="55"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="171">
         <f>A2+7</f>
         <v>46058</v>
@@ -8037,14 +8049,14 @@
         <v>2</v>
       </c>
       <c r="C3" s="170" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F3" s="75"/>
       <c r="G3" s="2"/>
       <c r="H3" s="26"/>
       <c r="I3" s="27"/>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="171">
         <f t="shared" ref="A4:A12" si="0">A3+7</f>
         <v>46065</v>
@@ -8061,7 +8073,7 @@
       <c r="H4" s="26"/>
       <c r="I4" s="27"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="171">
         <f t="shared" si="0"/>
         <v>46072</v>
@@ -8071,14 +8083,14 @@
         <v>4</v>
       </c>
       <c r="C5" s="170" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F5" s="75"/>
       <c r="G5" s="2"/>
       <c r="H5" s="26"/>
       <c r="I5" s="27"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="133">
         <f t="shared" si="0"/>
         <v>46079</v>
@@ -8095,7 +8107,7 @@
       <c r="H6" s="26"/>
       <c r="I6" s="27"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="133">
         <f t="shared" si="0"/>
         <v>46086</v>
@@ -8105,14 +8117,14 @@
         <v>6</v>
       </c>
       <c r="C7" s="134" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F7" s="75"/>
       <c r="G7" s="2"/>
       <c r="H7" s="26"/>
       <c r="I7" s="27"/>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="133">
         <f t="shared" si="0"/>
         <v>46093</v>
@@ -8129,7 +8141,7 @@
       <c r="H8" s="26"/>
       <c r="I8" s="27"/>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="133">
         <f t="shared" si="0"/>
         <v>46100</v>
@@ -8146,7 +8158,7 @@
       <c r="H9" s="26"/>
       <c r="I9" s="27"/>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="133">
         <f t="shared" si="0"/>
         <v>46107</v>
@@ -8163,7 +8175,7 @@
       <c r="H10" s="26"/>
       <c r="I10" s="27"/>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="133">
         <f t="shared" si="0"/>
         <v>46114</v>
@@ -8176,7 +8188,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="133">
         <f t="shared" si="0"/>
         <v>46121</v>
@@ -8189,7 +8201,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="133">
         <f t="shared" ref="A13:A14" si="3">A12+7</f>
         <v>46128</v>
@@ -8202,7 +8214,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="133">
         <f t="shared" si="3"/>
         <v>46135</v>
@@ -8215,12 +8227,12 @@
         <v>434</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="133"/>
       <c r="B15" s="134"/>
       <c r="C15" s="134"/>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="G16" s="26"/>
     </row>
   </sheetData>
@@ -8247,7 +8259,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2BB5C5F-5790-4A91-A6E8-8841719DA1FC}">
   <dimension ref="A2:I20"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" customWidth="1"/>
     <col min="2" max="2" width="9.140625" customWidth="1"/>
@@ -8259,17 +8271,17 @@
     <col min="9" max="9" width="64.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" ht="23.25">
+    <row r="2" spans="1:9" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A2" s="91" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="18.75">
+    <row r="3" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="79" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="37.5">
+    <row r="5" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A5" s="80" t="s">
         <v>3</v>
       </c>
@@ -8298,7 +8310,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="18.75">
+    <row r="6" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="92">
         <v>45694</v>
       </c>
@@ -8322,10 +8334,10 @@
       </c>
       <c r="H6" s="85"/>
       <c r="I6" s="84" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="18.75">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="83">
         <v>45708</v>
       </c>
@@ -8354,7 +8366,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="18.75">
+    <row r="8" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="83">
         <v>45722</v>
       </c>
@@ -8381,7 +8393,7 @@
       </c>
       <c r="I8" s="86"/>
     </row>
-    <row r="9" spans="1:9" ht="18.75">
+    <row r="9" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="83">
         <v>45735</v>
       </c>
@@ -8407,10 +8419,10 @@
         <v>206</v>
       </c>
       <c r="I9" s="86" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="18.75">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A10" s="83">
         <v>45744</v>
       </c>
@@ -8437,7 +8449,7 @@
       </c>
       <c r="I10" s="86"/>
     </row>
-    <row r="11" spans="1:9" ht="18.75">
+    <row r="11" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A11" s="83">
         <v>45750</v>
       </c>
@@ -8461,10 +8473,10 @@
       </c>
       <c r="H11" s="87"/>
       <c r="I11" s="86" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="18.75">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A12" s="83">
         <v>45758</v>
       </c>
@@ -8490,10 +8502,10 @@
         <v>31</v>
       </c>
       <c r="I12" s="86" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="18.75">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="83">
         <v>45764</v>
       </c>
@@ -8516,7 +8528,7 @@
       <c r="H13" s="87"/>
       <c r="I13" s="86"/>
     </row>
-    <row r="14" spans="1:9" ht="18.75">
+    <row r="14" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="88">
         <v>45771</v>
       </c>
@@ -8545,7 +8557,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="20" spans="8:8" ht="18.75">
+    <row r="20" spans="8:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="H20" s="79"/>
     </row>
   </sheetData>

</xml_diff>